<commit_message>
Add initial-order XA scenario and annual exports
</commit_message>
<xml_diff>
--- a/data/simulations/xa_fixed_v1/SIM_XA_FIXED_seed_20260809/competition_xlsx/SIM_XA_FIXED最终排名和破产信息.xlsx
+++ b/data/simulations/xa_fixed_v1/SIM_XA_FIXED_seed_20260809/competition_xlsx/SIM_XA_FIXED最终排名和破产信息.xlsx
@@ -480,17 +480,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED14</t>
+          <t>SIM_XA_FIXED24</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>415.5499999999998</v>
+        <v>371.5499999999998</v>
       </c>
       <c r="D2" t="n">
         <v>18</v>
       </c>
       <c r="E2" t="n">
-        <v>490</v>
+        <v>438</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -504,17 +504,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED10</t>
+          <t>SIM_XA_FIXED06</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>388.9999999999999</v>
+        <v>338</v>
       </c>
       <c r="D3" t="n">
         <v>18</v>
       </c>
       <c r="E3" t="n">
-        <v>459</v>
+        <v>399</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -528,17 +528,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED24</t>
+          <t>SIM_XA_FIXED25</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>335.9999999999999</v>
+        <v>309.9999999999999</v>
       </c>
       <c r="D4" t="n">
         <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>396</v>
+        <v>366</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -552,17 +552,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED21</t>
+          <t>SIM_XA_FIXED01</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="D5" t="n">
         <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>384</v>
+        <v>365</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -576,17 +576,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED02</t>
+          <t>SIM_XA_FIXED10</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>317.9999999999999</v>
+        <v>305</v>
       </c>
       <c r="D6" t="n">
         <v>18</v>
       </c>
       <c r="E6" t="n">
-        <v>375</v>
+        <v>360</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -600,17 +600,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED09</t>
+          <t>SIM_XA_FIXED20</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>310.9999999999999</v>
+        <v>300</v>
       </c>
       <c r="D7" t="n">
         <v>18</v>
       </c>
       <c r="E7" t="n">
-        <v>367</v>
+        <v>354</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -624,17 +624,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED15</t>
+          <t>SIM_XA_FIXED23</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>305</v>
+        <v>298.9999999999999</v>
       </c>
       <c r="D8" t="n">
         <v>18</v>
       </c>
       <c r="E8" t="n">
-        <v>360</v>
+        <v>353</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -648,17 +648,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED18</t>
+          <t>SIM_XA_FIXED26</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>300</v>
+        <v>298.9999999999999</v>
       </c>
       <c r="D9" t="n">
         <v>18</v>
       </c>
       <c r="E9" t="n">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -672,17 +672,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED25</t>
+          <t>SIM_XA_FIXED03</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>296</v>
+        <v>294.9999999999999</v>
       </c>
       <c r="D10" t="n">
         <v>18</v>
       </c>
       <c r="E10" t="n">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -696,17 +696,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED22</t>
+          <t>SIM_XA_FIXED27</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D11" t="n">
         <v>18</v>
       </c>
       <c r="E11" t="n">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -720,17 +720,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED06</t>
+          <t>SIM_XA_FIXED12</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D12" t="n">
         <v>18</v>
       </c>
       <c r="E12" t="n">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -744,17 +744,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED12</t>
+          <t>SIM_XA_FIXED18</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D13" t="n">
         <v>18</v>
       </c>
       <c r="E13" t="n">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -768,17 +768,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED20</t>
+          <t>SIM_XA_FIXED19</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D14" t="n">
         <v>18</v>
       </c>
       <c r="E14" t="n">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -792,17 +792,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED11</t>
+          <t>SIM_XA_FIXED16</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D15" t="n">
         <v>18</v>
       </c>
       <c r="E15" t="n">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -816,17 +816,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED17</t>
+          <t>SIM_XA_FIXED07</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D16" t="n">
         <v>18</v>
       </c>
       <c r="E16" t="n">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -840,17 +840,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED08</t>
+          <t>SIM_XA_FIXED22</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D17" t="n">
         <v>18</v>
       </c>
       <c r="E17" t="n">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -864,17 +864,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED19</t>
+          <t>SIM_XA_FIXED21</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>256.9999999999999</v>
+        <v>254</v>
       </c>
       <c r="D18" t="n">
         <v>18</v>
       </c>
       <c r="E18" t="n">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -888,17 +888,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED16</t>
+          <t>SIM_XA_FIXED09</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="D19" t="n">
         <v>18</v>
       </c>
       <c r="E19" t="n">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -912,17 +912,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED26</t>
+          <t>SIM_XA_FIXED05</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D20" t="n">
         <v>18</v>
       </c>
       <c r="E20" t="n">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -936,17 +936,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED23</t>
+          <t>SIM_XA_FIXED13</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="D21" t="n">
         <v>18</v>
       </c>
       <c r="E21" t="n">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -960,17 +960,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED03</t>
+          <t>SIM_XA_FIXED17</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D22" t="n">
         <v>18</v>
       </c>
       <c r="E22" t="n">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -984,7 +984,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED07</t>
+          <t>SIM_XA_FIXED04</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1008,17 +1008,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED27</t>
+          <t>SIM_XA_FIXED08</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D24" t="n">
         <v>18</v>
       </c>
       <c r="E24" t="n">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1032,17 +1032,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED04</t>
+          <t>SIM_XA_FIXED14</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D25" t="n">
         <v>18</v>
       </c>
       <c r="E25" t="n">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1056,17 +1056,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED05</t>
+          <t>SIM_XA_FIXED02</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D26" t="n">
         <v>18</v>
       </c>
       <c r="E26" t="n">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1080,17 +1080,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED13</t>
+          <t>SIM_XA_FIXED15</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D27" t="n">
         <v>18</v>
       </c>
       <c r="E27" t="n">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1104,17 +1104,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SIM_XA_FIXED01</t>
+          <t>SIM_XA_FIXED11</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D28" t="n">
         <v>18</v>
       </c>
       <c r="E28" t="n">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>

</xml_diff>